<commit_message>
Remove training data, models, and datasets from tracking - Add comprehensive .gitignore - Remove persons/ folder (training images) - Remove yolo_v9/datasets_yolov8/ folder - Remove .pt, .yml, .npy model files - Remove .avi video files Files remain locally but won't be pushed to GitHub
</commit_message>
<xml_diff>
--- a/class_timetable.xlsx
+++ b/class_timetable.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\giris\Desktop\AAS\opencv_attendence\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Roshan\OneDrive\Desktop\opencv_proj\opencv_attendence\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BBCF5892-63FF-4A7F-A0BD-6BD9504B557D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04564ABB-1EE8-43B8-A91F-C9810016FBFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -42,13 +42,13 @@
     <t>email</t>
   </si>
   <si>
-    <t>girishhrudhay@gmail.com</t>
-  </si>
-  <si>
     <t>Minor Project</t>
   </si>
   <si>
     <t>Padmini M S</t>
+  </si>
+  <si>
+    <t>rohananandgd1976@gmail.com@gmail.com</t>
   </si>
 </sst>
 </file>
@@ -406,13 +406,13 @@
         <v>0.54166666666666663</v>
       </c>
       <c r="C2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D2" t="s">
         <v>6</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" s="2" t="s">
         <v>7</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>5</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">

</xml_diff>